<commit_message>
Adaptar puntos 3, 5, 10, 11 y 12 y actualizar checklist
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NuMj3fWq11HABbrtni6hs7
</commit_message>
<xml_diff>
--- a/Checklist/Checklist de entregas - Rediseño Curricular 2026.xlsx
+++ b/Checklist/Checklist de entregas - Rediseño Curricular 2026.xlsx
@@ -2579,15 +2579,29 @@
       <c r="D28" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="E28" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F28" s="9"/>
-      <c r="G28" s="6"/>
-      <c r="H28" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I28" s="10"/>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I28" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Punto 3 Justificación (Comisión 1, versión consolidada). Adaptado en: 3. Justificación de la innovación curricular.docx</t>
+        </is>
+      </c>
       <c r="J28" s="6">
         <v>1</v>
       </c>
@@ -2605,15 +2619,29 @@
       <c r="D29" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="E29" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F29" s="9"/>
-      <c r="G29" s="6"/>
-      <c r="H29" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I29" s="10"/>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I29" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Punto 3 Justificación (Comisión 1, versión consolidada). Adaptado en: 3. Justificación de la innovación curricular.docx</t>
+        </is>
+      </c>
       <c r="J29" s="6">
         <v>1</v>
       </c>
@@ -2631,15 +2659,29 @@
       <c r="D30" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="E30" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F30" s="9"/>
-      <c r="G30" s="6"/>
-      <c r="H30" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I30" s="10"/>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I30" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Punto 3 Justificación (Comisión 1, versión consolidada). Adaptado en: 3. Justificación de la innovación curricular.docx</t>
+        </is>
+      </c>
       <c r="J30" s="6">
         <v>1</v>
       </c>
@@ -2657,15 +2699,29 @@
       <c r="D31" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="E31" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F31" s="9"/>
-      <c r="G31" s="6"/>
-      <c r="H31" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I31" s="10"/>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I31" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Punto 3 Justificación (Comisión 1, versión consolidada). Adaptado en: 3. Justificación de la innovación curricular.docx</t>
+        </is>
+      </c>
       <c r="J31" s="6">
         <v>1</v>
       </c>
@@ -2683,15 +2739,29 @@
       <c r="D32" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="E32" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F32" s="9"/>
-      <c r="G32" s="6"/>
-      <c r="H32" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I32" s="10"/>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I32" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Punto 3 Justificación (Comisión 1, versión consolidada). Adaptado en: 3. Justificación de la innovación curricular.docx</t>
+        </is>
+      </c>
       <c r="J32" s="6">
         <v>1</v>
       </c>
@@ -3847,15 +3917,29 @@
       <c r="D73" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="E73" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F73" s="9"/>
-      <c r="G73" s="6"/>
-      <c r="H73" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I73" s="10"/>
+      <c r="E73" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F73" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G73" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
+      <c r="H73" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I73" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Informe Subcomisión 5 Admisión, promoción y graduación. Adaptado en: 5. Admisión, promoción y graduación.docx</t>
+        </is>
+      </c>
       <c r="J73" s="6">
         <v>1</v>
       </c>
@@ -3873,15 +3957,29 @@
       <c r="D74" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="E74" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F74" s="9"/>
-      <c r="G74" s="6"/>
-      <c r="H74" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I74" s="10"/>
+      <c r="E74" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F74" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G74" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
+      <c r="H74" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I74" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Informe Subcomisión 5 Admisión, promoción y graduación. Adaptado en: 5. Admisión, promoción y graduación.docx</t>
+        </is>
+      </c>
       <c r="J74" s="6">
         <v>1</v>
       </c>
@@ -3899,15 +3997,29 @@
       <c r="D75" s="8" t="s">
         <v>196</v>
       </c>
-      <c r="E75" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F75" s="9"/>
-      <c r="G75" s="6"/>
-      <c r="H75" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I75" s="10"/>
+      <c r="E75" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F75" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G75" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
+      <c r="H75" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I75" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Informe Subcomisión 5 Admisión, promoción y graduación. Adaptado en: 5. Admisión, promoción y graduación.docx</t>
+        </is>
+      </c>
       <c r="J75" s="6">
         <v>1</v>
       </c>
@@ -3925,15 +4037,29 @@
       <c r="D76" s="8" t="s">
         <v>196</v>
       </c>
-      <c r="E76" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F76" s="9"/>
-      <c r="G76" s="6"/>
-      <c r="H76" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I76" s="10"/>
+      <c r="E76" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F76" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G76" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
+      <c r="H76" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I76" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Informe Subcomisión 5 Admisión, promoción y graduación. Adaptado en: 5. Admisión, promoción y graduación.docx</t>
+        </is>
+      </c>
       <c r="J76" s="6">
         <v>1</v>
       </c>
@@ -4507,15 +4633,29 @@
       <c r="D96" s="8" t="s">
         <v>245</v>
       </c>
-      <c r="E96" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F96" s="9"/>
-      <c r="G96" s="6"/>
-      <c r="H96" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I96" s="10"/>
+      <c r="E96" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F96" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G96" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
+      <c r="H96" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I96" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documento 10 Recursos educativos. Adaptado en: 10. Recursos educativos.docx</t>
+        </is>
+      </c>
       <c r="J96" s="6">
         <v>1</v>
       </c>
@@ -4533,15 +4673,29 @@
       <c r="D97" s="8" t="s">
         <v>245</v>
       </c>
-      <c r="E97" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F97" s="9"/>
-      <c r="G97" s="6"/>
-      <c r="H97" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I97" s="10"/>
+      <c r="E97" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F97" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G97" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
+      <c r="H97" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I97" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documento 10 Recursos educativos. Adaptado en: 10. Recursos educativos.docx</t>
+        </is>
+      </c>
       <c r="J97" s="6">
         <v>1</v>
       </c>
@@ -4559,15 +4713,29 @@
       <c r="D98" s="8" t="s">
         <v>245</v>
       </c>
-      <c r="E98" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F98" s="9"/>
-      <c r="G98" s="6"/>
-      <c r="H98" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I98" s="10"/>
+      <c r="E98" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F98" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G98" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
+      <c r="H98" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I98" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documento 10 Recursos educativos. Adaptado en: 10. Recursos educativos.docx</t>
+        </is>
+      </c>
       <c r="J98" s="6">
         <v>1</v>
       </c>
@@ -4585,15 +4753,29 @@
       <c r="D99" s="8" t="s">
         <v>245</v>
       </c>
-      <c r="E99" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F99" s="9"/>
-      <c r="G99" s="6"/>
-      <c r="H99" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I99" s="10"/>
+      <c r="E99" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F99" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G99" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
+      <c r="H99" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I99" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documento 10 Recursos educativos. Adaptado en: 10. Recursos educativos.docx</t>
+        </is>
+      </c>
       <c r="J99" s="6">
         <v>1</v>
       </c>
@@ -4611,15 +4793,29 @@
       <c r="D100" s="8" t="s">
         <v>256</v>
       </c>
-      <c r="E100" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F100" s="9"/>
-      <c r="G100" s="6"/>
-      <c r="H100" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I100" s="10"/>
+      <c r="E100" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F100" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G100" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
+      <c r="H100" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I100" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documento 10 Recursos educativos. Adaptado en: 10. Recursos educativos.docx</t>
+        </is>
+      </c>
       <c r="J100" s="6">
         <v>1</v>
       </c>
@@ -4637,15 +4833,29 @@
       <c r="D101" s="8" t="s">
         <v>256</v>
       </c>
-      <c r="E101" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F101" s="9"/>
-      <c r="G101" s="6"/>
-      <c r="H101" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I101" s="10"/>
+      <c r="E101" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F101" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G101" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
+      <c r="H101" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I101" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documento 10 Recursos educativos. Adaptado en: 10. Recursos educativos.docx</t>
+        </is>
+      </c>
       <c r="J101" s="6">
         <v>1</v>
       </c>
@@ -4663,15 +4873,29 @@
       <c r="D102" s="8" t="s">
         <v>256</v>
       </c>
-      <c r="E102" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F102" s="9"/>
-      <c r="G102" s="6"/>
-      <c r="H102" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I102" s="10"/>
+      <c r="E102" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F102" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G102" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
+      <c r="H102" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I102" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documento 10 Recursos educativos. Adaptado en: 10. Recursos educativos.docx</t>
+        </is>
+      </c>
       <c r="J102" s="6">
         <v>1</v>
       </c>
@@ -4689,15 +4913,29 @@
       <c r="D103" s="8" t="s">
         <v>256</v>
       </c>
-      <c r="E103" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F103" s="9"/>
-      <c r="G103" s="6"/>
-      <c r="H103" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I103" s="10"/>
+      <c r="E103" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F103" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G103" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
+      <c r="H103" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I103" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documento 10 Recursos educativos. Adaptado en: 10. Recursos educativos.docx</t>
+        </is>
+      </c>
       <c r="J103" s="6">
         <v>1</v>
       </c>
@@ -4715,15 +4953,29 @@
       <c r="D104" s="8" t="s">
         <v>256</v>
       </c>
-      <c r="E104" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F104" s="9"/>
-      <c r="G104" s="6"/>
-      <c r="H104" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I104" s="10"/>
+      <c r="E104" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F104" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G104" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
+      <c r="H104" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I104" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documento 10 Recursos educativos. Adaptado en: 10. Recursos educativos.docx</t>
+        </is>
+      </c>
       <c r="J104" s="6">
         <v>1</v>
       </c>
@@ -4741,15 +4993,29 @@
       <c r="D105" s="8" t="s">
         <v>268</v>
       </c>
-      <c r="E105" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F105" s="9"/>
-      <c r="G105" s="6"/>
-      <c r="H105" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I105" s="10"/>
+      <c r="E105" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F105" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G105" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
+      <c r="H105" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I105" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documento 10 Recursos educativos. Adaptado en: 10. Recursos educativos.docx</t>
+        </is>
+      </c>
       <c r="J105" s="6">
         <v>1</v>
       </c>
@@ -4767,15 +5033,29 @@
       <c r="D106" s="8" t="s">
         <v>268</v>
       </c>
-      <c r="E106" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F106" s="9"/>
-      <c r="G106" s="6"/>
-      <c r="H106" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I106" s="10"/>
+      <c r="E106" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F106" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G106" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
+      <c r="H106" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I106" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documento 10 Recursos educativos. Adaptado en: 10. Recursos educativos.docx</t>
+        </is>
+      </c>
       <c r="J106" s="6">
         <v>1</v>
       </c>
@@ -4793,15 +5073,29 @@
       <c r="D107" s="8" t="s">
         <v>268</v>
       </c>
-      <c r="E107" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F107" s="9"/>
-      <c r="G107" s="6"/>
-      <c r="H107" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I107" s="10"/>
+      <c r="E107" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F107" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G107" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
+      <c r="H107" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I107" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documento 10 Recursos educativos. Adaptado en: 10. Recursos educativos.docx</t>
+        </is>
+      </c>
       <c r="J107" s="6">
         <v>1</v>
       </c>
@@ -4849,15 +5143,29 @@
       <c r="D109" s="8" t="s">
         <v>275</v>
       </c>
-      <c r="E109" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F109" s="9"/>
-      <c r="G109" s="6"/>
-      <c r="H109" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I109" s="10"/>
+      <c r="E109" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F109" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G109" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
+      <c r="H109" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I109" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Informe Subcomisión 1.1 Implementación del Proyecto Curricular. Adaptado en: 11. Implementación del proyecto curricular.docx</t>
+        </is>
+      </c>
       <c r="J109" s="6">
         <v>1</v>
       </c>
@@ -4875,15 +5183,29 @@
       <c r="D110" s="8" t="s">
         <v>281</v>
       </c>
-      <c r="E110" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F110" s="9"/>
-      <c r="G110" s="6"/>
-      <c r="H110" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I110" s="10"/>
+      <c r="E110" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F110" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G110" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
+      <c r="H110" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I110" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Informe Subcomisión 1.1 Implementación del Proyecto Curricular. Adaptado en: 11. Implementación del proyecto curricular.docx</t>
+        </is>
+      </c>
       <c r="J110" s="6">
         <v>1</v>
       </c>
@@ -4901,15 +5223,29 @@
       <c r="D111" s="8" t="s">
         <v>281</v>
       </c>
-      <c r="E111" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F111" s="9"/>
-      <c r="G111" s="6"/>
-      <c r="H111" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I111" s="10"/>
+      <c r="E111" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F111" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G111" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
+      <c r="H111" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I111" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Informe Subcomisión 1.1 Implementación del Proyecto Curricular. Adaptado en: 11. Implementación del proyecto curricular.docx</t>
+        </is>
+      </c>
       <c r="J111" s="6">
         <v>1</v>
       </c>
@@ -4957,15 +5293,29 @@
       <c r="D113" s="8" t="s">
         <v>287</v>
       </c>
-      <c r="E113" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F113" s="9"/>
-      <c r="G113" s="6"/>
-      <c r="H113" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I113" s="10"/>
+      <c r="E113" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F113" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G113" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
+      <c r="H113" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I113" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documento 12 Evaluación curricular (Comisión 10). Adaptado en: 12. Evaluación curricular.docx</t>
+        </is>
+      </c>
       <c r="J113" s="6">
         <v>1</v>
       </c>
@@ -4983,15 +5333,29 @@
       <c r="D114" s="8" t="s">
         <v>292</v>
       </c>
-      <c r="E114" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F114" s="9"/>
-      <c r="G114" s="6"/>
-      <c r="H114" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I114" s="10"/>
+      <c r="E114" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F114" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G114" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
+      <c r="H114" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I114" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documento 12 Evaluación curricular (Comisión 10). Adaptado en: 12. Evaluación curricular.docx</t>
+        </is>
+      </c>
       <c r="J114" s="6">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
Adaptar punto 13 (base 2024) y registrar en checklist
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NuMj3fWq11HABbrtni6hs7
</commit_message>
<xml_diff>
--- a/Checklist/Checklist de entregas - Rediseño Curricular 2026.xlsx
+++ b/Checklist/Checklist de entregas - Rediseño Curricular 2026.xlsx
@@ -5403,15 +5403,29 @@
       <c r="D116" s="8" t="s">
         <v>296</v>
       </c>
-      <c r="E116" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F116" s="9"/>
-      <c r="G116" s="6"/>
-      <c r="H116" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I116" s="10"/>
+      <c r="E116" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F116" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G116" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
+      <c r="H116" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I116" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Base 2024: 13_01 Reglamentos académicos y administrativos. Adaptado en: 13. Reglamentación.docx. Informe de observaciones de la Subcomisión 13 en Contenido extra</t>
+        </is>
+      </c>
       <c r="J116" s="6">
         <v>1</v>
       </c>
@@ -5429,15 +5443,29 @@
       <c r="D117" s="8" t="s">
         <v>302</v>
       </c>
-      <c r="E117" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F117" s="9"/>
-      <c r="G117" s="6"/>
-      <c r="H117" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I117" s="10"/>
+      <c r="E117" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F117" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G117" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
+      <c r="H117" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I117" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Base 2024: 13_02 Reglamentación del centro de investigación. Adaptado en: 13. Reglamentación.docx. Informe de observaciones de la Subcomisión 13 en Contenido extra</t>
+        </is>
+      </c>
       <c r="J117" s="6">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
Checklist: agregar estado 'No aplica' que no cuenta en totales ni avance
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NuMj3fWq11HABbrtni6hs7
</commit_message>
<xml_diff>
--- a/Checklist/Checklist de entregas - Rediseño Curricular 2026.xlsx
+++ b/Checklist/Checklist de entregas - Rediseño Curricular 2026.xlsx
@@ -1102,7 +1102,7 @@
     <t>Resumen de avance por punto</t>
   </si>
   <si>
-    <t>Se calcula solo con los ítems entregables de la hoja Checklist.</t>
+    <t>Se calcula solo con los ítems entregables de la hoja Checklist. Los ítems marcados «No aplica» no cuentan en el total ni en el avance.</t>
   </si>
   <si>
     <t>Punto</t>
@@ -1291,7 +1291,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="7">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -1359,6 +1359,18 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FF595959"/>
+        <name val="Century Gothic"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD9D9D9"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1732,10 +1744,10 @@
         <v>15</v>
       </c>
       <c r="E5" s="3" t="str">
-        <f>IF(SUMPRODUCT(($J$6:$J$18=1)*($E$6:$E$18="Entregado"))=SUMPRODUCT(($J$6:$J$18=1)*1),"Completo",IF(SUMPRODUCT(($J$6:$J$18=1)*($E$6:$E$18="Pendiente"))=SUMPRODUCT(($J$6:$J$18=1)*1),"Pendiente","En proceso"))</f>
+        <f>IF(SUMPRODUCT(($J$6:$J$18=1)*($E$6:$E$18&lt;&gt;"No aplica"))=0,"No aplica",IF(SUMPRODUCT(($J$6:$J$18=1)*($E$6:$E$18="Entregado"))=SUMPRODUCT(($J$6:$J$18=1)*($E$6:$E$18&lt;&gt;"No aplica")),"Completo",IF(SUMPRODUCT(($J$6:$J$18=1)*($E$6:$E$18="Pendiente"))=SUMPRODUCT(($J$6:$J$18=1)*($E$6:$E$18&lt;&gt;"No aplica")),"Pendiente","En proceso")))</f>
       </c>
       <c r="F5" s="3" t="str">
-        <f>SUMPRODUCT(($J$6:$J$18=1)*($E$6:$E$18="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$6:$J$18=1)*1)</f>
+        <f>SUMPRODUCT(($J$6:$J$18=1)*($E$6:$E$18="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$6:$J$18=1)*($E$6:$E$18&lt;&gt;"No aplica"))</f>
       </c>
       <c r="G5" s="3" t="s">
         <v>16</v>
@@ -2268,10 +2280,10 @@
         <v>47</v>
       </c>
       <c r="E19" s="3" t="str">
-        <f>IF(SUMPRODUCT(($J$20:$J$26=1)*($E$20:$E$26="Entregado"))=SUMPRODUCT(($J$20:$J$26=1)*1),"Completo",IF(SUMPRODUCT(($J$20:$J$26=1)*($E$20:$E$26="Pendiente"))=SUMPRODUCT(($J$20:$J$26=1)*1),"Pendiente","En proceso"))</f>
+        <f>IF(SUMPRODUCT(($J$20:$J$26=1)*($E$20:$E$26&lt;&gt;"No aplica"))=0,"No aplica",IF(SUMPRODUCT(($J$20:$J$26=1)*($E$20:$E$26="Entregado"))=SUMPRODUCT(($J$20:$J$26=1)*($E$20:$E$26&lt;&gt;"No aplica")),"Completo",IF(SUMPRODUCT(($J$20:$J$26=1)*($E$20:$E$26="Pendiente"))=SUMPRODUCT(($J$20:$J$26=1)*($E$20:$E$26&lt;&gt;"No aplica")),"Pendiente","En proceso")))</f>
       </c>
       <c r="F19" s="3" t="str">
-        <f>SUMPRODUCT(($J$20:$J$26=1)*($E$20:$E$26="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$20:$J$26=1)*1)</f>
+        <f>SUMPRODUCT(($J$20:$J$26=1)*($E$20:$E$26="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$20:$J$26=1)*($E$20:$E$26&lt;&gt;"No aplica"))</f>
       </c>
       <c r="G19" s="3" t="s">
         <v>16</v>
@@ -2550,10 +2562,10 @@
         <v>65</v>
       </c>
       <c r="E27" s="3" t="str">
-        <f>IF(SUMPRODUCT(($J$28:$J$32=1)*($E$28:$E$32="Entregado"))=SUMPRODUCT(($J$28:$J$32=1)*1),"Completo",IF(SUMPRODUCT(($J$28:$J$32=1)*($E$28:$E$32="Pendiente"))=SUMPRODUCT(($J$28:$J$32=1)*1),"Pendiente","En proceso"))</f>
+        <f>IF(SUMPRODUCT(($J$28:$J$32=1)*($E$28:$E$32&lt;&gt;"No aplica"))=0,"No aplica",IF(SUMPRODUCT(($J$28:$J$32=1)*($E$28:$E$32="Entregado"))=SUMPRODUCT(($J$28:$J$32=1)*($E$28:$E$32&lt;&gt;"No aplica")),"Completo",IF(SUMPRODUCT(($J$28:$J$32=1)*($E$28:$E$32="Pendiente"))=SUMPRODUCT(($J$28:$J$32=1)*($E$28:$E$32&lt;&gt;"No aplica")),"Pendiente","En proceso")))</f>
       </c>
       <c r="F27" s="3" t="str">
-        <f>SUMPRODUCT(($J$28:$J$32=1)*($E$28:$E$32="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$28:$J$32=1)*1)</f>
+        <f>SUMPRODUCT(($J$28:$J$32=1)*($E$28:$E$32="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$28:$J$32=1)*($E$28:$E$32&lt;&gt;"No aplica"))</f>
       </c>
       <c r="G27" s="3" t="s">
         <v>16</v>
@@ -2780,10 +2792,10 @@
         <v>81</v>
       </c>
       <c r="E33" s="3" t="str">
-        <f>IF(SUMPRODUCT(($J$34:$J$71=1)*($E$34:$E$71="Entregado"))=SUMPRODUCT(($J$34:$J$71=1)*1),"Completo",IF(SUMPRODUCT(($J$34:$J$71=1)*($E$34:$E$71="Pendiente"))=SUMPRODUCT(($J$34:$J$71=1)*1),"Pendiente","En proceso"))</f>
+        <f>IF(SUMPRODUCT(($J$34:$J$71=1)*($E$34:$E$71&lt;&gt;"No aplica"))=0,"No aplica",IF(SUMPRODUCT(($J$34:$J$71=1)*($E$34:$E$71="Entregado"))=SUMPRODUCT(($J$34:$J$71=1)*($E$34:$E$71&lt;&gt;"No aplica")),"Completo",IF(SUMPRODUCT(($J$34:$J$71=1)*($E$34:$E$71="Pendiente"))=SUMPRODUCT(($J$34:$J$71=1)*($E$34:$E$71&lt;&gt;"No aplica")),"Pendiente","En proceso")))</f>
       </c>
       <c r="F33" s="3" t="str">
-        <f>SUMPRODUCT(($J$34:$J$71=1)*($E$34:$E$71="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$34:$J$71=1)*1)</f>
+        <f>SUMPRODUCT(($J$34:$J$71=1)*($E$34:$E$71="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$34:$J$71=1)*($E$34:$E$71&lt;&gt;"No aplica"))</f>
       </c>
       <c r="G33" s="3" t="s">
         <v>16</v>
@@ -2810,10 +2822,10 @@
         <v>81</v>
       </c>
       <c r="E34" s="11" t="str">
-        <f>IF(SUMPRODUCT(($J$35:$J$39=1)*($E$35:$E$39="Entregado"))=SUMPRODUCT(($J$35:$J$39=1)*1),"Completo",IF(SUMPRODUCT(($J$35:$J$39=1)*($E$35:$E$39="Pendiente"))=SUMPRODUCT(($J$35:$J$39=1)*1),"Pendiente","En proceso"))</f>
+        <f>IF(SUMPRODUCT(($J$35:$J$39=1)*($E$35:$E$39&lt;&gt;"No aplica"))=0,"No aplica",IF(SUMPRODUCT(($J$35:$J$39=1)*($E$35:$E$39="Entregado"))=SUMPRODUCT(($J$35:$J$39=1)*($E$35:$E$39&lt;&gt;"No aplica")),"Completo",IF(SUMPRODUCT(($J$35:$J$39=1)*($E$35:$E$39="Pendiente"))=SUMPRODUCT(($J$35:$J$39=1)*($E$35:$E$39&lt;&gt;"No aplica")),"Pendiente","En proceso")))</f>
       </c>
       <c r="F34" s="11" t="str">
-        <f>SUMPRODUCT(($J$35:$J$39=1)*($E$35:$E$39="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$35:$J$39=1)*1)</f>
+        <f>SUMPRODUCT(($J$35:$J$39=1)*($E$35:$E$39="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$35:$J$39=1)*($E$35:$E$39&lt;&gt;"No aplica"))</f>
       </c>
       <c r="G34" s="11" t="s">
         <v>16</v>
@@ -2970,10 +2982,10 @@
         <v>99</v>
       </c>
       <c r="E40" s="11" t="str">
-        <f>IF(SUMPRODUCT(($J$41:$J$47=1)*($E$41:$E$47="Entregado"))=SUMPRODUCT(($J$41:$J$47=1)*1),"Completo",IF(SUMPRODUCT(($J$41:$J$47=1)*($E$41:$E$47="Pendiente"))=SUMPRODUCT(($J$41:$J$47=1)*1),"Pendiente","En proceso"))</f>
+        <f>IF(SUMPRODUCT(($J$41:$J$47=1)*($E$41:$E$47&lt;&gt;"No aplica"))=0,"No aplica",IF(SUMPRODUCT(($J$41:$J$47=1)*($E$41:$E$47="Entregado"))=SUMPRODUCT(($J$41:$J$47=1)*($E$41:$E$47&lt;&gt;"No aplica")),"Completo",IF(SUMPRODUCT(($J$41:$J$47=1)*($E$41:$E$47="Pendiente"))=SUMPRODUCT(($J$41:$J$47=1)*($E$41:$E$47&lt;&gt;"No aplica")),"Pendiente","En proceso")))</f>
       </c>
       <c r="F40" s="11" t="str">
-        <f>SUMPRODUCT(($J$41:$J$47=1)*($E$41:$E$47="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$41:$J$47=1)*1)</f>
+        <f>SUMPRODUCT(($J$41:$J$47=1)*($E$41:$E$47="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$41:$J$47=1)*($E$41:$E$47&lt;&gt;"No aplica"))</f>
       </c>
       <c r="G40" s="11" t="s">
         <v>16</v>
@@ -3182,10 +3194,10 @@
         <v>117</v>
       </c>
       <c r="E48" s="11" t="str">
-        <f>IF(SUMPRODUCT(($J$49:$J$53=1)*($E$49:$E$53="Entregado"))=SUMPRODUCT(($J$49:$J$53=1)*1),"Completo",IF(SUMPRODUCT(($J$49:$J$53=1)*($E$49:$E$53="Pendiente"))=SUMPRODUCT(($J$49:$J$53=1)*1),"Pendiente","En proceso"))</f>
+        <f>IF(SUMPRODUCT(($J$49:$J$53=1)*($E$49:$E$53&lt;&gt;"No aplica"))=0,"No aplica",IF(SUMPRODUCT(($J$49:$J$53=1)*($E$49:$E$53="Entregado"))=SUMPRODUCT(($J$49:$J$53=1)*($E$49:$E$53&lt;&gt;"No aplica")),"Completo",IF(SUMPRODUCT(($J$49:$J$53=1)*($E$49:$E$53="Pendiente"))=SUMPRODUCT(($J$49:$J$53=1)*($E$49:$E$53&lt;&gt;"No aplica")),"Pendiente","En proceso")))</f>
       </c>
       <c r="F48" s="11" t="str">
-        <f>SUMPRODUCT(($J$49:$J$53=1)*($E$49:$E$53="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$49:$J$53=1)*1)</f>
+        <f>SUMPRODUCT(($J$49:$J$53=1)*($E$49:$E$53="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$49:$J$53=1)*($E$49:$E$53&lt;&gt;"No aplica"))</f>
       </c>
       <c r="G48" s="11" t="s">
         <v>16</v>
@@ -3412,10 +3424,10 @@
         <v>132</v>
       </c>
       <c r="E54" s="11" t="str">
-        <f>IF(SUMPRODUCT(($J$55:$J$58=1)*($E$55:$E$58="Entregado"))=SUMPRODUCT(($J$55:$J$58=1)*1),"Completo",IF(SUMPRODUCT(($J$55:$J$58=1)*($E$55:$E$58="Pendiente"))=SUMPRODUCT(($J$55:$J$58=1)*1),"Pendiente","En proceso"))</f>
+        <f>IF(SUMPRODUCT(($J$55:$J$58=1)*($E$55:$E$58&lt;&gt;"No aplica"))=0,"No aplica",IF(SUMPRODUCT(($J$55:$J$58=1)*($E$55:$E$58="Entregado"))=SUMPRODUCT(($J$55:$J$58=1)*($E$55:$E$58&lt;&gt;"No aplica")),"Completo",IF(SUMPRODUCT(($J$55:$J$58=1)*($E$55:$E$58="Pendiente"))=SUMPRODUCT(($J$55:$J$58=1)*($E$55:$E$58&lt;&gt;"No aplica")),"Pendiente","En proceso")))</f>
       </c>
       <c r="F54" s="11" t="str">
-        <f>SUMPRODUCT(($J$55:$J$58=1)*($E$55:$E$58="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$55:$J$58=1)*1)</f>
+        <f>SUMPRODUCT(($J$55:$J$58=1)*($E$55:$E$58="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$55:$J$58=1)*($E$55:$E$58&lt;&gt;"No aplica"))</f>
       </c>
       <c r="G54" s="11" t="s">
         <v>16</v>
@@ -3546,10 +3558,10 @@
         <v>143</v>
       </c>
       <c r="E59" s="11" t="str">
-        <f>IF(SUMPRODUCT(($J$60:$J$68=1)*($E$60:$E$68="Entregado"))=SUMPRODUCT(($J$60:$J$68=1)*1),"Completo",IF(SUMPRODUCT(($J$60:$J$68=1)*($E$60:$E$68="Pendiente"))=SUMPRODUCT(($J$60:$J$68=1)*1),"Pendiente","En proceso"))</f>
+        <f>IF(SUMPRODUCT(($J$60:$J$68=1)*($E$60:$E$68&lt;&gt;"No aplica"))=0,"No aplica",IF(SUMPRODUCT(($J$60:$J$68=1)*($E$60:$E$68="Entregado"))=SUMPRODUCT(($J$60:$J$68=1)*($E$60:$E$68&lt;&gt;"No aplica")),"Completo",IF(SUMPRODUCT(($J$60:$J$68=1)*($E$60:$E$68="Pendiente"))=SUMPRODUCT(($J$60:$J$68=1)*($E$60:$E$68&lt;&gt;"No aplica")),"Pendiente","En proceso")))</f>
       </c>
       <c r="F59" s="11" t="str">
-        <f>SUMPRODUCT(($J$60:$J$68=1)*($E$60:$E$68="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$60:$J$68=1)*1)</f>
+        <f>SUMPRODUCT(($J$60:$J$68=1)*($E$60:$E$68="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$60:$J$68=1)*($E$60:$E$68&lt;&gt;"No aplica"))</f>
       </c>
       <c r="G59" s="11" t="s">
         <v>16</v>
@@ -3888,10 +3900,10 @@
         <v>188</v>
       </c>
       <c r="E72" s="3" t="str">
-        <f>IF(SUMPRODUCT(($J$73:$J$76=1)*($E$73:$E$76="Entregado"))=SUMPRODUCT(($J$73:$J$76=1)*1),"Completo",IF(SUMPRODUCT(($J$73:$J$76=1)*($E$73:$E$76="Pendiente"))=SUMPRODUCT(($J$73:$J$76=1)*1),"Pendiente","En proceso"))</f>
+        <f>IF(SUMPRODUCT(($J$73:$J$76=1)*($E$73:$E$76&lt;&gt;"No aplica"))=0,"No aplica",IF(SUMPRODUCT(($J$73:$J$76=1)*($E$73:$E$76="Entregado"))=SUMPRODUCT(($J$73:$J$76=1)*($E$73:$E$76&lt;&gt;"No aplica")),"Completo",IF(SUMPRODUCT(($J$73:$J$76=1)*($E$73:$E$76="Pendiente"))=SUMPRODUCT(($J$73:$J$76=1)*($E$73:$E$76&lt;&gt;"No aplica")),"Pendiente","En proceso")))</f>
       </c>
       <c r="F72" s="3" t="str">
-        <f>SUMPRODUCT(($J$73:$J$76=1)*($E$73:$E$76="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$73:$J$76=1)*1)</f>
+        <f>SUMPRODUCT(($J$73:$J$76=1)*($E$73:$E$76="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$73:$J$76=1)*($E$73:$E$76&lt;&gt;"No aplica"))</f>
       </c>
       <c r="G72" s="3" t="s">
         <v>16</v>
@@ -4078,10 +4090,10 @@
         <v>201</v>
       </c>
       <c r="E77" s="3" t="str">
-        <f>IF(SUMPRODUCT(($J$78:$J$79=1)*($E$78:$E$79="Entregado"))=SUMPRODUCT(($J$78:$J$79=1)*1),"Completo",IF(SUMPRODUCT(($J$78:$J$79=1)*($E$78:$E$79="Pendiente"))=SUMPRODUCT(($J$78:$J$79=1)*1),"Pendiente","En proceso"))</f>
+        <f>IF(SUMPRODUCT(($J$78:$J$79=1)*($E$78:$E$79&lt;&gt;"No aplica"))=0,"No aplica",IF(SUMPRODUCT(($J$78:$J$79=1)*($E$78:$E$79="Entregado"))=SUMPRODUCT(($J$78:$J$79=1)*($E$78:$E$79&lt;&gt;"No aplica")),"Completo",IF(SUMPRODUCT(($J$78:$J$79=1)*($E$78:$E$79="Pendiente"))=SUMPRODUCT(($J$78:$J$79=1)*($E$78:$E$79&lt;&gt;"No aplica")),"Pendiente","En proceso")))</f>
       </c>
       <c r="F77" s="3" t="str">
-        <f>SUMPRODUCT(($J$78:$J$79=1)*($E$78:$E$79="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$78:$J$79=1)*1)</f>
+        <f>SUMPRODUCT(($J$78:$J$79=1)*($E$78:$E$79="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$78:$J$79=1)*($E$78:$E$79&lt;&gt;"No aplica"))</f>
       </c>
       <c r="G77" s="3" t="s">
         <v>16</v>
@@ -4188,10 +4200,10 @@
         <v>209</v>
       </c>
       <c r="E80" s="3" t="str">
-        <f>IF(SUMPRODUCT(($J$81:$J$82=1)*($E$81:$E$82="Entregado"))=SUMPRODUCT(($J$81:$J$82=1)*1),"Completo",IF(SUMPRODUCT(($J$81:$J$82=1)*($E$81:$E$82="Pendiente"))=SUMPRODUCT(($J$81:$J$82=1)*1),"Pendiente","En proceso"))</f>
+        <f>IF(SUMPRODUCT(($J$81:$J$82=1)*($E$81:$E$82&lt;&gt;"No aplica"))=0,"No aplica",IF(SUMPRODUCT(($J$81:$J$82=1)*($E$81:$E$82="Entregado"))=SUMPRODUCT(($J$81:$J$82=1)*($E$81:$E$82&lt;&gt;"No aplica")),"Completo",IF(SUMPRODUCT(($J$81:$J$82=1)*($E$81:$E$82="Pendiente"))=SUMPRODUCT(($J$81:$J$82=1)*($E$81:$E$82&lt;&gt;"No aplica")),"Pendiente","En proceso")))</f>
       </c>
       <c r="F80" s="3" t="str">
-        <f>SUMPRODUCT(($J$81:$J$82=1)*($E$81:$E$82="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$81:$J$82=1)*1)</f>
+        <f>SUMPRODUCT(($J$81:$J$82=1)*($E$81:$E$82="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$81:$J$82=1)*($E$81:$E$82&lt;&gt;"No aplica"))</f>
       </c>
       <c r="G80" s="3" t="s">
         <v>16</v>
@@ -4270,10 +4282,10 @@
         <v>132</v>
       </c>
       <c r="E83" s="3" t="str">
-        <f>IF(SUMPRODUCT(($J$84:$J$89=1)*($E$84:$E$89="Entregado"))=SUMPRODUCT(($J$84:$J$89=1)*1),"Completo",IF(SUMPRODUCT(($J$84:$J$89=1)*($E$84:$E$89="Pendiente"))=SUMPRODUCT(($J$84:$J$89=1)*1),"Pendiente","En proceso"))</f>
+        <f>IF(SUMPRODUCT(($J$84:$J$89=1)*($E$84:$E$89&lt;&gt;"No aplica"))=0,"No aplica",IF(SUMPRODUCT(($J$84:$J$89=1)*($E$84:$E$89="Entregado"))=SUMPRODUCT(($J$84:$J$89=1)*($E$84:$E$89&lt;&gt;"No aplica")),"Completo",IF(SUMPRODUCT(($J$84:$J$89=1)*($E$84:$E$89="Pendiente"))=SUMPRODUCT(($J$84:$J$89=1)*($E$84:$E$89&lt;&gt;"No aplica")),"Pendiente","En proceso")))</f>
       </c>
       <c r="F83" s="3" t="str">
-        <f>SUMPRODUCT(($J$84:$J$89=1)*($E$84:$E$89="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$84:$J$89=1)*1)</f>
+        <f>SUMPRODUCT(($J$84:$J$89=1)*($E$84:$E$89="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$84:$J$89=1)*($E$84:$E$89&lt;&gt;"No aplica"))</f>
       </c>
       <c r="G83" s="3" t="s">
         <v>16</v>
@@ -4456,10 +4468,10 @@
         <v>231</v>
       </c>
       <c r="E90" s="3" t="str">
-        <f>IF(SUMPRODUCT(($J$91:$J$94=1)*($E$91:$E$94="Entregado"))=SUMPRODUCT(($J$91:$J$94=1)*1),"Completo",IF(SUMPRODUCT(($J$91:$J$94=1)*($E$91:$E$94="Pendiente"))=SUMPRODUCT(($J$91:$J$94=1)*1),"Pendiente","En proceso"))</f>
+        <f>IF(SUMPRODUCT(($J$91:$J$94=1)*($E$91:$E$94&lt;&gt;"No aplica"))=0,"No aplica",IF(SUMPRODUCT(($J$91:$J$94=1)*($E$91:$E$94="Entregado"))=SUMPRODUCT(($J$91:$J$94=1)*($E$91:$E$94&lt;&gt;"No aplica")),"Completo",IF(SUMPRODUCT(($J$91:$J$94=1)*($E$91:$E$94="Pendiente"))=SUMPRODUCT(($J$91:$J$94=1)*($E$91:$E$94&lt;&gt;"No aplica")),"Pendiente","En proceso")))</f>
       </c>
       <c r="F90" s="3" t="str">
-        <f>SUMPRODUCT(($J$91:$J$94=1)*($E$91:$E$94="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$91:$J$94=1)*1)</f>
+        <f>SUMPRODUCT(($J$91:$J$94=1)*($E$91:$E$94="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$91:$J$94=1)*($E$91:$E$94&lt;&gt;"No aplica"))</f>
       </c>
       <c r="G90" s="3" t="s">
         <v>16</v>
@@ -4604,10 +4616,10 @@
         <v>245</v>
       </c>
       <c r="E95" s="3" t="str">
-        <f>IF(SUMPRODUCT(($J$96:$J$107=1)*($E$96:$E$107="Entregado"))=SUMPRODUCT(($J$96:$J$107=1)*1),"Completo",IF(SUMPRODUCT(($J$96:$J$107=1)*($E$96:$E$107="Pendiente"))=SUMPRODUCT(($J$96:$J$107=1)*1),"Pendiente","En proceso"))</f>
+        <f>IF(SUMPRODUCT(($J$96:$J$107=1)*($E$96:$E$107&lt;&gt;"No aplica"))=0,"No aplica",IF(SUMPRODUCT(($J$96:$J$107=1)*($E$96:$E$107="Entregado"))=SUMPRODUCT(($J$96:$J$107=1)*($E$96:$E$107&lt;&gt;"No aplica")),"Completo",IF(SUMPRODUCT(($J$96:$J$107=1)*($E$96:$E$107="Pendiente"))=SUMPRODUCT(($J$96:$J$107=1)*($E$96:$E$107&lt;&gt;"No aplica")),"Pendiente","En proceso")))</f>
       </c>
       <c r="F95" s="3" t="str">
-        <f>SUMPRODUCT(($J$96:$J$107=1)*($E$96:$E$107="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$96:$J$107=1)*1)</f>
+        <f>SUMPRODUCT(($J$96:$J$107=1)*($E$96:$E$107="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$96:$J$107=1)*($E$96:$E$107&lt;&gt;"No aplica"))</f>
       </c>
       <c r="G95" s="3" t="s">
         <v>16</v>
@@ -5114,10 +5126,10 @@
         <v>275</v>
       </c>
       <c r="E108" s="3" t="str">
-        <f>IF(SUMPRODUCT(($J$109:$J$111=1)*($E$109:$E$111="Entregado"))=SUMPRODUCT(($J$109:$J$111=1)*1),"Completo",IF(SUMPRODUCT(($J$109:$J$111=1)*($E$109:$E$111="Pendiente"))=SUMPRODUCT(($J$109:$J$111=1)*1),"Pendiente","En proceso"))</f>
+        <f>IF(SUMPRODUCT(($J$109:$J$111=1)*($E$109:$E$111&lt;&gt;"No aplica"))=0,"No aplica",IF(SUMPRODUCT(($J$109:$J$111=1)*($E$109:$E$111="Entregado"))=SUMPRODUCT(($J$109:$J$111=1)*($E$109:$E$111&lt;&gt;"No aplica")),"Completo",IF(SUMPRODUCT(($J$109:$J$111=1)*($E$109:$E$111="Pendiente"))=SUMPRODUCT(($J$109:$J$111=1)*($E$109:$E$111&lt;&gt;"No aplica")),"Pendiente","En proceso")))</f>
       </c>
       <c r="F108" s="3" t="str">
-        <f>SUMPRODUCT(($J$109:$J$111=1)*($E$109:$E$111="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$109:$J$111=1)*1)</f>
+        <f>SUMPRODUCT(($J$109:$J$111=1)*($E$109:$E$111="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$109:$J$111=1)*($E$109:$E$111&lt;&gt;"No aplica"))</f>
       </c>
       <c r="G108" s="3" t="s">
         <v>16</v>
@@ -5264,10 +5276,10 @@
         <v>287</v>
       </c>
       <c r="E112" s="3" t="str">
-        <f>IF(SUMPRODUCT(($J$113:$J$114=1)*($E$113:$E$114="Entregado"))=SUMPRODUCT(($J$113:$J$114=1)*1),"Completo",IF(SUMPRODUCT(($J$113:$J$114=1)*($E$113:$E$114="Pendiente"))=SUMPRODUCT(($J$113:$J$114=1)*1),"Pendiente","En proceso"))</f>
+        <f>IF(SUMPRODUCT(($J$113:$J$114=1)*($E$113:$E$114&lt;&gt;"No aplica"))=0,"No aplica",IF(SUMPRODUCT(($J$113:$J$114=1)*($E$113:$E$114="Entregado"))=SUMPRODUCT(($J$113:$J$114=1)*($E$113:$E$114&lt;&gt;"No aplica")),"Completo",IF(SUMPRODUCT(($J$113:$J$114=1)*($E$113:$E$114="Pendiente"))=SUMPRODUCT(($J$113:$J$114=1)*($E$113:$E$114&lt;&gt;"No aplica")),"Pendiente","En proceso")))</f>
       </c>
       <c r="F112" s="3" t="str">
-        <f>SUMPRODUCT(($J$113:$J$114=1)*($E$113:$E$114="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$113:$J$114=1)*1)</f>
+        <f>SUMPRODUCT(($J$113:$J$114=1)*($E$113:$E$114="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$113:$J$114=1)*($E$113:$E$114&lt;&gt;"No aplica"))</f>
       </c>
       <c r="G112" s="3" t="s">
         <v>16</v>
@@ -5374,10 +5386,10 @@
         <v>296</v>
       </c>
       <c r="E115" s="3" t="str">
-        <f>IF(SUMPRODUCT(($J$116:$J$117=1)*($E$116:$E$117="Entregado"))=SUMPRODUCT(($J$116:$J$117=1)*1),"Completo",IF(SUMPRODUCT(($J$116:$J$117=1)*($E$116:$E$117="Pendiente"))=SUMPRODUCT(($J$116:$J$117=1)*1),"Pendiente","En proceso"))</f>
+        <f>IF(SUMPRODUCT(($J$116:$J$117=1)*($E$116:$E$117&lt;&gt;"No aplica"))=0,"No aplica",IF(SUMPRODUCT(($J$116:$J$117=1)*($E$116:$E$117="Entregado"))=SUMPRODUCT(($J$116:$J$117=1)*($E$116:$E$117&lt;&gt;"No aplica")),"Completo",IF(SUMPRODUCT(($J$116:$J$117=1)*($E$116:$E$117="Pendiente"))=SUMPRODUCT(($J$116:$J$117=1)*($E$116:$E$117&lt;&gt;"No aplica")),"Pendiente","En proceso")))</f>
       </c>
       <c r="F115" s="3" t="str">
-        <f>SUMPRODUCT(($J$116:$J$117=1)*($E$116:$E$117="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$116:$J$117=1)*1)</f>
+        <f>SUMPRODUCT(($J$116:$J$117=1)*($E$116:$E$117="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$116:$J$117=1)*($E$116:$E$117&lt;&gt;"No aplica"))</f>
       </c>
       <c r="G115" s="3" t="s">
         <v>16</v>
@@ -5484,10 +5496,10 @@
         <v>306</v>
       </c>
       <c r="E118" s="3" t="str">
-        <f>IF(SUMPRODUCT(($J$119:$J$127=1)*($E$119:$E$127="Entregado"))=SUMPRODUCT(($J$119:$J$127=1)*1),"Completo",IF(SUMPRODUCT(($J$119:$J$127=1)*($E$119:$E$127="Pendiente"))=SUMPRODUCT(($J$119:$J$127=1)*1),"Pendiente","En proceso"))</f>
+        <f>IF(SUMPRODUCT(($J$119:$J$127=1)*($E$119:$E$127&lt;&gt;"No aplica"))=0,"No aplica",IF(SUMPRODUCT(($J$119:$J$127=1)*($E$119:$E$127="Entregado"))=SUMPRODUCT(($J$119:$J$127=1)*($E$119:$E$127&lt;&gt;"No aplica")),"Completo",IF(SUMPRODUCT(($J$119:$J$127=1)*($E$119:$E$127="Pendiente"))=SUMPRODUCT(($J$119:$J$127=1)*($E$119:$E$127&lt;&gt;"No aplica")),"Pendiente","En proceso")))</f>
       </c>
       <c r="F118" s="3" t="str">
-        <f>SUMPRODUCT(($J$119:$J$127=1)*($E$119:$E$127="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$119:$J$127=1)*1)</f>
+        <f>SUMPRODUCT(($J$119:$J$127=1)*($E$119:$E$127="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$119:$J$127=1)*($E$119:$E$127&lt;&gt;"No aplica"))</f>
       </c>
       <c r="G118" s="3" t="s">
         <v>16</v>
@@ -5818,10 +5830,10 @@
         <v>329</v>
       </c>
       <c r="E128" s="3" t="str">
-        <f>IF(SUMPRODUCT(($J$129:$J$133=1)*($E$129:$E$133="Entregado"))=SUMPRODUCT(($J$129:$J$133=1)*1),"Completo",IF(SUMPRODUCT(($J$129:$J$133=1)*($E$129:$E$133="Pendiente"))=SUMPRODUCT(($J$129:$J$133=1)*1),"Pendiente","En proceso"))</f>
+        <f>IF(SUMPRODUCT(($J$129:$J$133=1)*($E$129:$E$133&lt;&gt;"No aplica"))=0,"No aplica",IF(SUMPRODUCT(($J$129:$J$133=1)*($E$129:$E$133="Entregado"))=SUMPRODUCT(($J$129:$J$133=1)*($E$129:$E$133&lt;&gt;"No aplica")),"Completo",IF(SUMPRODUCT(($J$129:$J$133=1)*($E$129:$E$133="Pendiente"))=SUMPRODUCT(($J$129:$J$133=1)*($E$129:$E$133&lt;&gt;"No aplica")),"Pendiente","En proceso")))</f>
       </c>
       <c r="F128" s="3" t="str">
-        <f>SUMPRODUCT(($J$129:$J$133=1)*($E$129:$E$133="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$129:$J$133=1)*1)</f>
+        <f>SUMPRODUCT(($J$129:$J$133=1)*($E$129:$E$133="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$129:$J$133=1)*($E$129:$E$133&lt;&gt;"No aplica"))</f>
       </c>
       <c r="G128" s="3" t="s">
         <v>16</v>
@@ -5978,10 +5990,10 @@
         <v>344</v>
       </c>
       <c r="E134" s="3" t="str">
-        <f>IF(SUMPRODUCT(($J$135:$J$137=1)*($E$135:$E$137="Entregado"))=SUMPRODUCT(($J$135:$J$137=1)*1),"Completo",IF(SUMPRODUCT(($J$135:$J$137=1)*($E$135:$E$137="Pendiente"))=SUMPRODUCT(($J$135:$J$137=1)*1),"Pendiente","En proceso"))</f>
+        <f>IF(SUMPRODUCT(($J$135:$J$137=1)*($E$135:$E$137&lt;&gt;"No aplica"))=0,"No aplica",IF(SUMPRODUCT(($J$135:$J$137=1)*($E$135:$E$137="Entregado"))=SUMPRODUCT(($J$135:$J$137=1)*($E$135:$E$137&lt;&gt;"No aplica")),"Completo",IF(SUMPRODUCT(($J$135:$J$137=1)*($E$135:$E$137="Pendiente"))=SUMPRODUCT(($J$135:$J$137=1)*($E$135:$E$137&lt;&gt;"No aplica")),"Pendiente","En proceso")))</f>
       </c>
       <c r="F134" s="3" t="str">
-        <f>SUMPRODUCT(($J$135:$J$137=1)*($E$135:$E$137="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$135:$J$137=1)*1)</f>
+        <f>SUMPRODUCT(($J$135:$J$137=1)*($E$135:$E$137="Entregado"))&amp;" de "&amp;SUMPRODUCT(($J$135:$J$137=1)*($E$135:$E$137&lt;&gt;"No aplica"))</f>
       </c>
       <c r="G134" s="3" t="s">
         <v>16</v>
@@ -6090,6 +6102,9 @@
     <cfRule type="expression" dxfId="1" priority="5">
       <formula>E5="Observado"</formula>
     </cfRule>
+    <cfRule type="expression" dxfId="6" priority="7">
+      <formula>E5="No aplica"</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H5:H137">
     <cfRule type="expression" dxfId="0" priority="6">
@@ -6098,7 +6113,7 @@
   </conditionalFormatting>
   <dataValidations count="4">
     <dataValidation type="list" showErrorMessage="1" errorTitle="Estado" error="Elija un estado de la lista." sqref="E6:E18 E135:E137 E28:E32 E35:E39 E20:E26 E49:E53 E55:E58 E60:E71 E73:E76 E78:E79 E81:E82 E84:E89 E91:E94 E96:E107 E109:E111 E113:E114 E116:E117 E119:E127 E129:E133 E41:E47" xr:uid="{00000000-0002-0000-0000-000000000000}">
-      <formula1>"Pendiente,Entregado,Parcial,Observado"</formula1>
+      <formula1>"Pendiente,Entregado,Parcial,Observado,No aplica"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="G6:G18 G20:G26 G28:G32 G35:G39 G135:G137 G49:G53 G55:G58 G60:G71 G73:G76 G78:G79 G81:G82 G84:G89 G91:G94 G96:G107 G109:G111 G113:G114 G116:G117 G119:G127 G129:G133 G41:G47" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Word,PDF,Excel,PowerPoint,Otro"</formula1>
@@ -6124,7 +6139,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -6134,6 +6149,7 @@
     <col min="5" max="5" width="11" customWidth="1"/>
     <col min="6" max="7" width="12" customWidth="1"/>
     <col min="8" max="8" width="11" customWidth="1"/>
+    <col min="9" max="9" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -6146,7 +6162,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="25.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" ht="25.2" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>355</v>
       </c>
@@ -6171,8 +6187,13 @@
       <c r="H4" s="3" t="s">
         <v>362</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="6">
         <v>1</v>
       </c>
@@ -6180,7 +6201,7 @@
         <v>13</v>
       </c>
       <c r="C5" s="6">
-        <f>COUNTIFS(Checklist!$A$5:$A$137,"1.*",Checklist!$J$5:$J$137,1)</f>
+        <f>COUNTIFS(Checklist!$A$5:$A$137,"1.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"&lt;&gt;No aplica")</f>
       </c>
       <c r="D5" s="6">
         <f>COUNTIFS(Checklist!$A$5:$A$137,"1.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"Entregado")</f>
@@ -6195,10 +6216,13 @@
         <f>COUNTIFS(Checklist!$A$5:$A$137,"1.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"Pendiente")</f>
       </c>
       <c r="H5" s="20">
-        <f t="shared" ref="H5:H21" si="0">IF(C5=0,0,D5/C5)</f>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+        <f t="shared" ref="H5:H21" si="0">IF(C5=0,IF(I5&gt;0,1,0),D5/C5)</f>
+      </c>
+      <c r="I5" s="6">
+        <f>COUNTIFS(Checklist!$A$5:$A$137,"1.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"No aplica")</f>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="6">
         <v>2</v>
       </c>
@@ -6206,7 +6230,7 @@
         <v>46</v>
       </c>
       <c r="C6" s="6">
-        <f>COUNTIFS(Checklist!$A$5:$A$137,"2.*",Checklist!$J$5:$J$137,1)</f>
+        <f>COUNTIFS(Checklist!$A$5:$A$137,"2.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"&lt;&gt;No aplica")</f>
       </c>
       <c r="D6" s="6">
         <f>COUNTIFS(Checklist!$A$5:$A$137,"2.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"Entregado")</f>
@@ -6223,8 +6247,11 @@
       <c r="H6" s="20">
         <f t="shared" si="0"/>
       </c>
-    </row>
-    <row r="7" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="I6" s="6">
+        <f>COUNTIFS(Checklist!$A$5:$A$137,"2.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"No aplica")</f>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A7" s="6">
         <v>3</v>
       </c>
@@ -6232,7 +6259,7 @@
         <v>63</v>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS(Checklist!$A$5:$A$137,"3.*",Checklist!$J$5:$J$137,1)</f>
+        <f>COUNTIFS(Checklist!$A$5:$A$137,"3.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"&lt;&gt;No aplica")</f>
       </c>
       <c r="D7" s="6">
         <f>COUNTIFS(Checklist!$A$5:$A$137,"3.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"Entregado")</f>
@@ -6249,8 +6276,11 @@
       <c r="H7" s="20">
         <f t="shared" si="0"/>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I7" s="6">
+        <f>COUNTIFS(Checklist!$A$5:$A$137,"3.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"No aplica")</f>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="6">
         <v>4</v>
       </c>
@@ -6258,7 +6288,7 @@
         <v>79</v>
       </c>
       <c r="C8" s="6">
-        <f>COUNTIFS(Checklist!$A$5:$A$137,"4.*",Checklist!$J$5:$J$137,1)</f>
+        <f>COUNTIFS(Checklist!$A$5:$A$137,"4.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"&lt;&gt;No aplica")</f>
       </c>
       <c r="D8" s="6">
         <f>COUNTIFS(Checklist!$A$5:$A$137,"4.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"Entregado")</f>
@@ -6275,8 +6305,11 @@
       <c r="H8" s="20">
         <f t="shared" si="0"/>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I8" s="6">
+        <f>COUNTIFS(Checklist!$A$5:$A$137,"4.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"No aplica")</f>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="6">
         <v>5</v>
       </c>
@@ -6284,7 +6317,7 @@
         <v>186</v>
       </c>
       <c r="C9" s="6">
-        <f>COUNTIFS(Checklist!$A$5:$A$137,"5.*",Checklist!$J$5:$J$137,1)</f>
+        <f>COUNTIFS(Checklist!$A$5:$A$137,"5.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"&lt;&gt;No aplica")</f>
       </c>
       <c r="D9" s="6">
         <f>COUNTIFS(Checklist!$A$5:$A$137,"5.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"Entregado")</f>
@@ -6301,8 +6334,11 @@
       <c r="H9" s="20">
         <f t="shared" si="0"/>
       </c>
-    </row>
-    <row r="10" spans="1:8" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="I9" s="6">
+        <f>COUNTIFS(Checklist!$A$5:$A$137,"5.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"No aplica")</f>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A10" s="6">
         <v>6</v>
       </c>
@@ -6310,7 +6346,7 @@
         <v>200</v>
       </c>
       <c r="C10" s="6">
-        <f>COUNTIFS(Checklist!$A$5:$A$137,"6.*",Checklist!$J$5:$J$137,1)</f>
+        <f>COUNTIFS(Checklist!$A$5:$A$137,"6.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"&lt;&gt;No aplica")</f>
       </c>
       <c r="D10" s="6">
         <f>COUNTIFS(Checklist!$A$5:$A$137,"6.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"Entregado")</f>
@@ -6327,8 +6363,11 @@
       <c r="H10" s="20">
         <f t="shared" si="0"/>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I10" s="6">
+        <f>COUNTIFS(Checklist!$A$5:$A$137,"6.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"No aplica")</f>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="6">
         <v>7</v>
       </c>
@@ -6336,7 +6375,7 @@
         <v>207</v>
       </c>
       <c r="C11" s="6">
-        <f>COUNTIFS(Checklist!$A$5:$A$137,"7.*",Checklist!$J$5:$J$137,1)</f>
+        <f>COUNTIFS(Checklist!$A$5:$A$137,"7.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"&lt;&gt;No aplica")</f>
       </c>
       <c r="D11" s="6">
         <f>COUNTIFS(Checklist!$A$5:$A$137,"7.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"Entregado")</f>
@@ -6353,8 +6392,11 @@
       <c r="H11" s="20">
         <f t="shared" si="0"/>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I11" s="6">
+        <f>COUNTIFS(Checklist!$A$5:$A$137,"7.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"No aplica")</f>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="6">
         <v>8</v>
       </c>
@@ -6362,7 +6404,7 @@
         <v>215</v>
       </c>
       <c r="C12" s="6">
-        <f>COUNTIFS(Checklist!$A$5:$A$137,"8.*",Checklist!$J$5:$J$137,1)</f>
+        <f>COUNTIFS(Checklist!$A$5:$A$137,"8.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"&lt;&gt;No aplica")</f>
       </c>
       <c r="D12" s="6">
         <f>COUNTIFS(Checklist!$A$5:$A$137,"8.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"Entregado")</f>
@@ -6379,8 +6421,11 @@
       <c r="H12" s="20">
         <f t="shared" si="0"/>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I12" s="6">
+        <f>COUNTIFS(Checklist!$A$5:$A$137,"8.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"No aplica")</f>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="6">
         <v>9</v>
       </c>
@@ -6388,7 +6433,7 @@
         <v>229</v>
       </c>
       <c r="C13" s="6">
-        <f>COUNTIFS(Checklist!$A$5:$A$137,"9.*",Checklist!$J$5:$J$137,1)</f>
+        <f>COUNTIFS(Checklist!$A$5:$A$137,"9.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"&lt;&gt;No aplica")</f>
       </c>
       <c r="D13" s="6">
         <f>COUNTIFS(Checklist!$A$5:$A$137,"9.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"Entregado")</f>
@@ -6405,8 +6450,11 @@
       <c r="H13" s="20">
         <f t="shared" si="0"/>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I13" s="6">
+        <f>COUNTIFS(Checklist!$A$5:$A$137,"9.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"No aplica")</f>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="6">
         <v>10</v>
       </c>
@@ -6414,7 +6462,7 @@
         <v>243</v>
       </c>
       <c r="C14" s="6">
-        <f>COUNTIFS(Checklist!$A$5:$A$137,"10.*",Checklist!$J$5:$J$137,1)</f>
+        <f>COUNTIFS(Checklist!$A$5:$A$137,"10.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"&lt;&gt;No aplica")</f>
       </c>
       <c r="D14" s="6">
         <f>COUNTIFS(Checklist!$A$5:$A$137,"10.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"Entregado")</f>
@@ -6431,8 +6479,11 @@
       <c r="H14" s="20">
         <f t="shared" si="0"/>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I14" s="6">
+        <f>COUNTIFS(Checklist!$A$5:$A$137,"10.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"No aplica")</f>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="6">
         <v>11</v>
       </c>
@@ -6440,7 +6491,7 @@
         <v>274</v>
       </c>
       <c r="C15" s="6">
-        <f>COUNTIFS(Checklist!$A$5:$A$137,"11.*",Checklist!$J$5:$J$137,1)</f>
+        <f>COUNTIFS(Checklist!$A$5:$A$137,"11.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"&lt;&gt;No aplica")</f>
       </c>
       <c r="D15" s="6">
         <f>COUNTIFS(Checklist!$A$5:$A$137,"11.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"Entregado")</f>
@@ -6457,8 +6508,11 @@
       <c r="H15" s="20">
         <f t="shared" si="0"/>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I15" s="6">
+        <f>COUNTIFS(Checklist!$A$5:$A$137,"11.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"No aplica")</f>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="6">
         <v>12</v>
       </c>
@@ -6466,7 +6520,7 @@
         <v>285</v>
       </c>
       <c r="C16" s="6">
-        <f>COUNTIFS(Checklist!$A$5:$A$137,"12.*",Checklist!$J$5:$J$137,1)</f>
+        <f>COUNTIFS(Checklist!$A$5:$A$137,"12.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"&lt;&gt;No aplica")</f>
       </c>
       <c r="D16" s="6">
         <f>COUNTIFS(Checklist!$A$5:$A$137,"12.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"Entregado")</f>
@@ -6483,8 +6537,11 @@
       <c r="H16" s="20">
         <f t="shared" si="0"/>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I16" s="6">
+        <f>COUNTIFS(Checklist!$A$5:$A$137,"12.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"No aplica")</f>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="6">
         <v>13</v>
       </c>
@@ -6492,7 +6549,7 @@
         <v>294</v>
       </c>
       <c r="C17" s="6">
-        <f>COUNTIFS(Checklist!$A$5:$A$137,"13.*",Checklist!$J$5:$J$137,1)</f>
+        <f>COUNTIFS(Checklist!$A$5:$A$137,"13.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"&lt;&gt;No aplica")</f>
       </c>
       <c r="D17" s="6">
         <f>COUNTIFS(Checklist!$A$5:$A$137,"13.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"Entregado")</f>
@@ -6509,8 +6566,11 @@
       <c r="H17" s="20">
         <f t="shared" si="0"/>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I17" s="6">
+        <f>COUNTIFS(Checklist!$A$5:$A$137,"13.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"No aplica")</f>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="6">
         <v>14</v>
       </c>
@@ -6518,7 +6578,7 @@
         <v>304</v>
       </c>
       <c r="C18" s="6">
-        <f>COUNTIFS(Checklist!$A$5:$A$137,"14.*",Checklist!$J$5:$J$137,1)</f>
+        <f>COUNTIFS(Checklist!$A$5:$A$137,"14.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"&lt;&gt;No aplica")</f>
       </c>
       <c r="D18" s="6">
         <f>COUNTIFS(Checklist!$A$5:$A$137,"14.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"Entregado")</f>
@@ -6535,8 +6595,11 @@
       <c r="H18" s="20">
         <f t="shared" si="0"/>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I18" s="6">
+        <f>COUNTIFS(Checklist!$A$5:$A$137,"14.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"No aplica")</f>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="6">
         <v>15</v>
       </c>
@@ -6544,7 +6607,7 @@
         <v>327</v>
       </c>
       <c r="C19" s="6">
-        <f>COUNTIFS(Checklist!$A$5:$A$137,"15.*",Checklist!$J$5:$J$137,1)</f>
+        <f>COUNTIFS(Checklist!$A$5:$A$137,"15.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"&lt;&gt;No aplica")</f>
       </c>
       <c r="D19" s="6">
         <f>COUNTIFS(Checklist!$A$5:$A$137,"15.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"Entregado")</f>
@@ -6561,8 +6624,11 @@
       <c r="H19" s="20">
         <f t="shared" si="0"/>
       </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I19" s="6">
+        <f>COUNTIFS(Checklist!$A$5:$A$137,"15.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"No aplica")</f>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="6">
         <v>16</v>
       </c>
@@ -6570,7 +6636,7 @@
         <v>343</v>
       </c>
       <c r="C20" s="6">
-        <f>COUNTIFS(Checklist!$A$5:$A$137,"16.*",Checklist!$J$5:$J$137,1)</f>
+        <f>COUNTIFS(Checklist!$A$5:$A$137,"16.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"&lt;&gt;No aplica")</f>
       </c>
       <c r="D20" s="6">
         <f>COUNTIFS(Checklist!$A$5:$A$137,"16.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"Entregado")</f>
@@ -6587,8 +6653,11 @@
       <c r="H20" s="20">
         <f t="shared" si="0"/>
       </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I20" s="6">
+        <f>COUNTIFS(Checklist!$A$5:$A$137,"16.*",Checklist!$J$5:$J$137,1,Checklist!$E$5:$E$137,"No aplica")</f>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="21"/>
       <c r="B21" s="22" t="s">
         <v>363</v>
@@ -6610,6 +6679,9 @@
       </c>
       <c r="H21" s="23">
         <f t="shared" si="0"/>
+      </c>
+      <c r="I21" s="21">
+        <f>SUM(I5:I20)</f>
       </c>
     </row>
   </sheetData>

</xml_diff>